<commit_message>
added script to run
</commit_message>
<xml_diff>
--- a/generic_node_optimization/userData/Summary.xlsx
+++ b/generic_node_optimization/userData/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE56"/>
+  <dimension ref="A1:AE58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6137,6 +6137,208 @@
       <c r="AE56" t="inlineStr">
         <is>
           <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111151612-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>206374471.7594043</v>
+      </c>
+      <c r="B57" t="n">
+        <v>123144411.5805673</v>
+      </c>
+      <c r="C57" t="n">
+        <v>31475491.71627041</v>
+      </c>
+      <c r="D57" t="n">
+        <v>44761469.74045806</v>
+      </c>
+      <c r="E57" t="n">
+        <v>214.917069864332</v>
+      </c>
+      <c r="F57" t="n">
+        <v>167905881.3210253</v>
+      </c>
+      <c r="G57" t="n">
+        <v>31475706.63334028</v>
+      </c>
+      <c r="H57" t="n">
+        <v>3774464.228086495</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" t="n">
+        <v>206374471.7594043</v>
+      </c>
+      <c r="N57" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>0</v>
+      </c>
+      <c r="R57" t="n">
+        <v>0</v>
+      </c>
+      <c r="S57" t="n">
+        <v>0</v>
+      </c>
+      <c r="T57" t="n">
+        <v>0</v>
+      </c>
+      <c r="U57" t="n">
+        <v>0</v>
+      </c>
+      <c r="V57" t="n">
+        <v>5.383000135421753</v>
+      </c>
+      <c r="W57" t="n">
+        <v>205159922.6600288</v>
+      </c>
+      <c r="X57" t="n">
+        <v>206374471.7594043</v>
+      </c>
+      <c r="Y57" t="n">
+        <v>1214549.099375427</v>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB57" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD57" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE57" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111152447-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>206374471.7594043</v>
+      </c>
+      <c r="B58" t="n">
+        <v>123144411.5805673</v>
+      </c>
+      <c r="C58" t="n">
+        <v>31475491.71627041</v>
+      </c>
+      <c r="D58" t="n">
+        <v>44761469.74045806</v>
+      </c>
+      <c r="E58" t="n">
+        <v>214.917069864332</v>
+      </c>
+      <c r="F58" t="n">
+        <v>167905881.3210253</v>
+      </c>
+      <c r="G58" t="n">
+        <v>31475706.63334028</v>
+      </c>
+      <c r="H58" t="n">
+        <v>3774464.228086495</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" t="n">
+        <v>206374471.7594043</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0</v>
+      </c>
+      <c r="P58" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>0</v>
+      </c>
+      <c r="R58" t="n">
+        <v>0</v>
+      </c>
+      <c r="S58" t="n">
+        <v>0</v>
+      </c>
+      <c r="T58" t="n">
+        <v>0</v>
+      </c>
+      <c r="U58" t="n">
+        <v>0</v>
+      </c>
+      <c r="V58" t="n">
+        <v>4.096999883651733</v>
+      </c>
+      <c r="W58" t="n">
+        <v>205159922.6600288</v>
+      </c>
+      <c r="X58" t="n">
+        <v>206374471.7594043</v>
+      </c>
+      <c r="Y58" t="n">
+        <v>1214549.099375427</v>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB58" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC58" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD58" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE58" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111153138-1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added network_minim option and cost og h2 constraint
</commit_message>
<xml_diff>
--- a/generic_node_optimization/userData/Summary.xlsx
+++ b/generic_node_optimization/userData/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE60"/>
+  <dimension ref="A1:AE67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6541,6 +6541,713 @@
       <c r="AE60" t="inlineStr">
         <is>
           <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111154344-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>613955210997.3405</v>
+      </c>
+      <c r="B61" t="n">
+        <v>417316658.4252779</v>
+      </c>
+      <c r="C61" t="n">
+        <v>20681485.05257106</v>
+      </c>
+      <c r="D61" t="n">
+        <v>151570000</v>
+      </c>
+      <c r="E61" t="n">
+        <v>29.3516706498561</v>
+      </c>
+      <c r="F61" t="n">
+        <v>568886658.4252779</v>
+      </c>
+      <c r="G61" t="n">
+        <v>20681514.40424171</v>
+      </c>
+      <c r="H61" t="n">
+        <v>3942898.380649222</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="n">
+        <v>0</v>
+      </c>
+      <c r="M61" t="n">
+        <v>613955210997.3405</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>0</v>
+      </c>
+      <c r="R61" t="n">
+        <v>0</v>
+      </c>
+      <c r="S61" t="n">
+        <v>0</v>
+      </c>
+      <c r="T61" t="n">
+        <v>0</v>
+      </c>
+      <c r="U61" t="n">
+        <v>0</v>
+      </c>
+      <c r="V61" t="n">
+        <v>2.874000072479248</v>
+      </c>
+      <c r="W61" t="n">
+        <v>20681514.40424171</v>
+      </c>
+      <c r="X61" t="n">
+        <v>20681514.40424171</v>
+      </c>
+      <c r="Y61" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB61" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC61" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD61" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE61" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111163630-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>613968451700.2793</v>
+      </c>
+      <c r="B62" t="n">
+        <v>417316658.4252779</v>
+      </c>
+      <c r="C62" t="n">
+        <v>27762693.60450269</v>
+      </c>
+      <c r="D62" t="n">
+        <v>151570000</v>
+      </c>
+      <c r="E62" t="n">
+        <v>214.8927791529596</v>
+      </c>
+      <c r="F62" t="n">
+        <v>568886658.4252779</v>
+      </c>
+      <c r="G62" t="n">
+        <v>27762908.49728184</v>
+      </c>
+      <c r="H62" t="n">
+        <v>10102207.22640333</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0</v>
+      </c>
+      <c r="M62" t="n">
+        <v>613968451700.2793</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>0</v>
+      </c>
+      <c r="R62" t="n">
+        <v>0</v>
+      </c>
+      <c r="S62" t="n">
+        <v>0</v>
+      </c>
+      <c r="T62" t="n">
+        <v>0</v>
+      </c>
+      <c r="U62" t="n">
+        <v>0</v>
+      </c>
+      <c r="V62" t="n">
+        <v>8.276000022888184</v>
+      </c>
+      <c r="W62" t="n">
+        <v>27762908.49728184</v>
+      </c>
+      <c r="X62" t="n">
+        <v>27762908.49728184</v>
+      </c>
+      <c r="Y62" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB62" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC62" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD62" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE62" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111164050-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>613968452453.5601</v>
+      </c>
+      <c r="B63" t="n">
+        <v>417316658.4252779</v>
+      </c>
+      <c r="C63" t="n">
+        <v>27762693.6045027</v>
+      </c>
+      <c r="D63" t="n">
+        <v>151570000</v>
+      </c>
+      <c r="E63" t="n">
+        <v>214.8927791529596</v>
+      </c>
+      <c r="F63" t="n">
+        <v>568886658.4252779</v>
+      </c>
+      <c r="G63" t="n">
+        <v>27762908.49728186</v>
+      </c>
+      <c r="H63" t="n">
+        <v>10102960.50716176</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="n">
+        <v>0</v>
+      </c>
+      <c r="M63" t="n">
+        <v>613968452453.5601</v>
+      </c>
+      <c r="N63" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>0</v>
+      </c>
+      <c r="R63" t="n">
+        <v>0</v>
+      </c>
+      <c r="S63" t="n">
+        <v>0</v>
+      </c>
+      <c r="T63" t="n">
+        <v>0</v>
+      </c>
+      <c r="U63" t="n">
+        <v>0</v>
+      </c>
+      <c r="V63" t="n">
+        <v>6.940999984741211</v>
+      </c>
+      <c r="W63" t="n">
+        <v>27762908.49728185</v>
+      </c>
+      <c r="X63" t="n">
+        <v>27762908.49728186</v>
+      </c>
+      <c r="Y63" t="n">
+        <v>3.725290298461914e-09</v>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB63" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD63" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE63" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111164226-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>672145153.0212166</v>
+      </c>
+      <c r="B64" t="n">
+        <v>399689766.8748745</v>
+      </c>
+      <c r="C64" t="n">
+        <v>27762693.6045027</v>
+      </c>
+      <c r="D64" t="n">
+        <v>145170000</v>
+      </c>
+      <c r="E64" t="n">
+        <v>214.8927791529596</v>
+      </c>
+      <c r="F64" t="n">
+        <v>544859766.8748745</v>
+      </c>
+      <c r="G64" t="n">
+        <v>27762908.49728186</v>
+      </c>
+      <c r="H64" t="n">
+        <v>10099407.83225391</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M64" t="n">
+        <v>672145153.0212166</v>
+      </c>
+      <c r="N64" t="n">
+        <v>0</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0</v>
+      </c>
+      <c r="P64" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>0</v>
+      </c>
+      <c r="R64" t="n">
+        <v>0</v>
+      </c>
+      <c r="S64" t="n">
+        <v>0</v>
+      </c>
+      <c r="T64" t="n">
+        <v>0</v>
+      </c>
+      <c r="U64" t="n">
+        <v>0</v>
+      </c>
+      <c r="V64" t="n">
+        <v>8.197999954223633</v>
+      </c>
+      <c r="W64" t="n">
+        <v>27762908.49728186</v>
+      </c>
+      <c r="X64" t="n">
+        <v>27762908.49728186</v>
+      </c>
+      <c r="Y64" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB64" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC64" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD64" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE64" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111173509-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>647369029.914942</v>
+      </c>
+      <c r="B65" t="n">
+        <v>399689766.8748745</v>
+      </c>
+      <c r="C65" t="n">
+        <v>15649634.32569422</v>
+      </c>
+      <c r="D65" t="n">
+        <v>145170000</v>
+      </c>
+      <c r="E65" t="n">
+        <v>3.543129979401723</v>
+      </c>
+      <c r="F65" t="n">
+        <v>544859766.8748745</v>
+      </c>
+      <c r="G65" t="n">
+        <v>15649637.8688242</v>
+      </c>
+      <c r="H65" t="n">
+        <v>389198.310378673</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" t="n">
+        <v>0</v>
+      </c>
+      <c r="M65" t="n">
+        <v>647369029.914942</v>
+      </c>
+      <c r="N65" t="n">
+        <v>0</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0</v>
+      </c>
+      <c r="P65" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>0</v>
+      </c>
+      <c r="R65" t="n">
+        <v>0</v>
+      </c>
+      <c r="S65" t="n">
+        <v>0</v>
+      </c>
+      <c r="T65" t="n">
+        <v>0</v>
+      </c>
+      <c r="U65" t="n">
+        <v>0</v>
+      </c>
+      <c r="V65" t="n">
+        <v>0.3629999160766602</v>
+      </c>
+      <c r="W65" t="n">
+        <v>15507259.85426485</v>
+      </c>
+      <c r="X65" t="n">
+        <v>15649637.8688242</v>
+      </c>
+      <c r="Y65" t="n">
+        <v>142378.014559349</v>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB65" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC65" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD65" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE65" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111173803-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>647369029.914942</v>
+      </c>
+      <c r="B66" t="n">
+        <v>399689766.8748745</v>
+      </c>
+      <c r="C66" t="n">
+        <v>15649634.32569422</v>
+      </c>
+      <c r="D66" t="n">
+        <v>145170000</v>
+      </c>
+      <c r="E66" t="n">
+        <v>3.543129979401723</v>
+      </c>
+      <c r="F66" t="n">
+        <v>544859766.8748745</v>
+      </c>
+      <c r="G66" t="n">
+        <v>15649637.8688242</v>
+      </c>
+      <c r="H66" t="n">
+        <v>389198.310378673</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" t="n">
+        <v>647369029.914942</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>0</v>
+      </c>
+      <c r="R66" t="n">
+        <v>0</v>
+      </c>
+      <c r="S66" t="n">
+        <v>0</v>
+      </c>
+      <c r="T66" t="n">
+        <v>0</v>
+      </c>
+      <c r="U66" t="n">
+        <v>0</v>
+      </c>
+      <c r="V66" t="n">
+        <v>0.3399999141693115</v>
+      </c>
+      <c r="W66" t="n">
+        <v>15507259.85426485</v>
+      </c>
+      <c r="X66" t="n">
+        <v>15649637.8688242</v>
+      </c>
+      <c r="Y66" t="n">
+        <v>142378.014559349</v>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB66" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD66" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE66" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111174156-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>647369029.914942</v>
+      </c>
+      <c r="B67" t="n">
+        <v>399689766.8748745</v>
+      </c>
+      <c r="C67" t="n">
+        <v>15649634.32569422</v>
+      </c>
+      <c r="D67" t="n">
+        <v>145170000</v>
+      </c>
+      <c r="E67" t="n">
+        <v>3.543129979401723</v>
+      </c>
+      <c r="F67" t="n">
+        <v>544859766.8748745</v>
+      </c>
+      <c r="G67" t="n">
+        <v>15649637.8688242</v>
+      </c>
+      <c r="H67" t="n">
+        <v>389198.310378673</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" t="n">
+        <v>0</v>
+      </c>
+      <c r="M67" t="n">
+        <v>647369029.914942</v>
+      </c>
+      <c r="N67" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0</v>
+      </c>
+      <c r="P67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>0</v>
+      </c>
+      <c r="R67" t="n">
+        <v>0</v>
+      </c>
+      <c r="S67" t="n">
+        <v>0</v>
+      </c>
+      <c r="T67" t="n">
+        <v>0</v>
+      </c>
+      <c r="U67" t="n">
+        <v>0</v>
+      </c>
+      <c r="V67" t="n">
+        <v>0.3739998340606689</v>
+      </c>
+      <c r="W67" t="n">
+        <v>15507259.85426485</v>
+      </c>
+      <c r="X67" t="n">
+        <v>15649637.8688242</v>
+      </c>
+      <c r="Y67" t="n">
+        <v>142378.014559349</v>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB67" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC67" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD67" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE67" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251111174434-1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added network distance minimization weighted with size
</commit_message>
<xml_diff>
--- a/generic_node_optimization/userData/Summary.xlsx
+++ b/generic_node_optimization/userData/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE75"/>
+  <dimension ref="A1:AE81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8056,6 +8056,612 @@
       <c r="AE75" t="inlineStr">
         <is>
           <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251112103547-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>381384585.5992096</v>
+      </c>
+      <c r="B76" t="n">
+        <v>33946254.17293455</v>
+      </c>
+      <c r="C76" t="n">
+        <v>2233469.94771684</v>
+      </c>
+      <c r="D76" t="n">
+        <v>12329506.84931507</v>
+      </c>
+      <c r="E76" t="n">
+        <v>5327.95720283495</v>
+      </c>
+      <c r="F76" t="n">
+        <v>46275761.02224962</v>
+      </c>
+      <c r="G76" t="n">
+        <v>2238797.904919675</v>
+      </c>
+      <c r="H76" t="n">
+        <v>306007331.6601691</v>
+      </c>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" t="n">
+        <v>381384585.5992096</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>0</v>
+      </c>
+      <c r="R76" t="n">
+        <v>0</v>
+      </c>
+      <c r="S76" t="n">
+        <v>0</v>
+      </c>
+      <c r="T76" t="n">
+        <v>0</v>
+      </c>
+      <c r="U76" t="n">
+        <v>0</v>
+      </c>
+      <c r="V76" t="n">
+        <v>5800.637000083923</v>
+      </c>
+      <c r="W76" t="n">
+        <v>2238797.904919675</v>
+      </c>
+      <c r="X76" t="n">
+        <v>2238797.904919675</v>
+      </c>
+      <c r="Y76" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB76" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC76" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD76" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE76" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251112131158-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>379631807.1061973</v>
+      </c>
+      <c r="B77" t="n">
+        <v>33946254.17293455</v>
+      </c>
+      <c r="C77" t="n">
+        <v>2233469.947716841</v>
+      </c>
+      <c r="D77" t="n">
+        <v>12329506.84931507</v>
+      </c>
+      <c r="E77" t="n">
+        <v>5327.957202834951</v>
+      </c>
+      <c r="F77" t="n">
+        <v>46275761.02224962</v>
+      </c>
+      <c r="G77" t="n">
+        <v>2238797.904919676</v>
+      </c>
+      <c r="H77" t="n">
+        <v>305410144.0942782</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" t="n">
+        <v>379631807.1061973</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>0</v>
+      </c>
+      <c r="R77" t="n">
+        <v>0</v>
+      </c>
+      <c r="S77" t="n">
+        <v>0</v>
+      </c>
+      <c r="T77" t="n">
+        <v>0</v>
+      </c>
+      <c r="U77" t="n">
+        <v>0</v>
+      </c>
+      <c r="V77" t="n">
+        <v>10459.66599988937</v>
+      </c>
+      <c r="W77" t="n">
+        <v>2238797.904919676</v>
+      </c>
+      <c r="X77" t="n">
+        <v>2238797.904919676</v>
+      </c>
+      <c r="Y77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB77" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC77" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD77" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE77" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251112150014-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>366341234.2137824</v>
+      </c>
+      <c r="B78" t="n">
+        <v>33946254.17293455</v>
+      </c>
+      <c r="C78" t="n">
+        <v>2233469.947716841</v>
+      </c>
+      <c r="D78" t="n">
+        <v>12329506.84931507</v>
+      </c>
+      <c r="E78" t="n">
+        <v>5327.957202834953</v>
+      </c>
+      <c r="F78" t="n">
+        <v>46275761.02224962</v>
+      </c>
+      <c r="G78" t="n">
+        <v>2238797.904919676</v>
+      </c>
+      <c r="H78" t="n">
+        <v>304430468.8466861</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" t="n">
+        <v>366341234.2137824</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0</v>
+      </c>
+      <c r="P78" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>0</v>
+      </c>
+      <c r="R78" t="n">
+        <v>0</v>
+      </c>
+      <c r="S78" t="n">
+        <v>0</v>
+      </c>
+      <c r="T78" t="n">
+        <v>0</v>
+      </c>
+      <c r="U78" t="n">
+        <v>0</v>
+      </c>
+      <c r="V78" t="n">
+        <v>9521.098000049591</v>
+      </c>
+      <c r="W78" t="n">
+        <v>2238797.904919676</v>
+      </c>
+      <c r="X78" t="n">
+        <v>2238797.904919676</v>
+      </c>
+      <c r="Y78" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB78" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC78" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD78" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE78" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251112180712-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>340460041.1379905</v>
+      </c>
+      <c r="B79" t="n">
+        <v>19635592.6556833</v>
+      </c>
+      <c r="C79" t="n">
+        <v>2233469.947716841</v>
+      </c>
+      <c r="D79" t="n">
+        <v>7133568.971557268</v>
+      </c>
+      <c r="E79" t="n">
+        <v>5327.957202834951</v>
+      </c>
+      <c r="F79" t="n">
+        <v>26769161.62724057</v>
+      </c>
+      <c r="G79" t="n">
+        <v>2238797.904919676</v>
+      </c>
+      <c r="H79" t="n">
+        <v>304099912.0577021</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" t="n">
+        <v>340460041.1379905</v>
+      </c>
+      <c r="N79" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" t="n">
+        <v>0</v>
+      </c>
+      <c r="P79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>0</v>
+      </c>
+      <c r="R79" t="n">
+        <v>0</v>
+      </c>
+      <c r="S79" t="n">
+        <v>0</v>
+      </c>
+      <c r="T79" t="n">
+        <v>0</v>
+      </c>
+      <c r="U79" t="n">
+        <v>0</v>
+      </c>
+      <c r="V79" t="n">
+        <v>13757.07699990273</v>
+      </c>
+      <c r="W79" t="n">
+        <v>2238797.904919676</v>
+      </c>
+      <c r="X79" t="n">
+        <v>2238797.904919676</v>
+      </c>
+      <c r="Y79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB79" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD79" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE79" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251112215137-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>321545594.4080989</v>
+      </c>
+      <c r="B80" t="n">
+        <v>17053674.77170376</v>
+      </c>
+      <c r="C80" t="n">
+        <v>2257953.471532406</v>
+      </c>
+      <c r="D80" t="n">
+        <v>6196122.083186078</v>
+      </c>
+      <c r="E80" t="n">
+        <v>5030.224255521372</v>
+      </c>
+      <c r="F80" t="n">
+        <v>23249796.85488984</v>
+      </c>
+      <c r="G80" t="n">
+        <v>2262983.695787928</v>
+      </c>
+      <c r="H80" t="n">
+        <v>294897479.7701125</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" t="n">
+        <v>321545594.4080989</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" t="n">
+        <v>0</v>
+      </c>
+      <c r="S80" t="n">
+        <v>0</v>
+      </c>
+      <c r="T80" t="n">
+        <v>0</v>
+      </c>
+      <c r="U80" t="n">
+        <v>0</v>
+      </c>
+      <c r="V80" t="n">
+        <v>26259.58299994469</v>
+      </c>
+      <c r="W80" t="n">
+        <v>2250937.341614723</v>
+      </c>
+      <c r="X80" t="n">
+        <v>2262983.695787928</v>
+      </c>
+      <c r="Y80" t="n">
+        <v>12046.3541732044</v>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB80" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD80" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE80" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113093541-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>321545594.408095</v>
+      </c>
+      <c r="B81" t="n">
+        <v>18682951.1203878</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1625939.143093377</v>
+      </c>
+      <c r="D81" t="n">
+        <v>6787682.352437004</v>
+      </c>
+      <c r="E81" t="n">
+        <v>5671.691255362147</v>
+      </c>
+      <c r="F81" t="n">
+        <v>25470633.4728248</v>
+      </c>
+      <c r="G81" t="n">
+        <v>1631610.83434874</v>
+      </c>
+      <c r="H81" t="n">
+        <v>293499314.4052019</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" t="n">
+        <v>321545594.408095</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>0</v>
+      </c>
+      <c r="R81" t="n">
+        <v>0</v>
+      </c>
+      <c r="S81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T81" t="n">
+        <v>0</v>
+      </c>
+      <c r="U81" t="n">
+        <v>0</v>
+      </c>
+      <c r="V81" t="n">
+        <v>164.8179998397827</v>
+      </c>
+      <c r="W81" t="n">
+        <v>1631544.54332544</v>
+      </c>
+      <c r="X81" t="n">
+        <v>1631610.83434874</v>
+      </c>
+      <c r="Y81" t="n">
+        <v>66.29102329933085</v>
+      </c>
+      <c r="Z81" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB81" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD81" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE81" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113170115-1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updates to new optimization
</commit_message>
<xml_diff>
--- a/generic_node_optimization/userData/Summary.xlsx
+++ b/generic_node_optimization/userData/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE81"/>
+  <dimension ref="A1:AE104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8662,6 +8662,2329 @@
       <c r="AE81" t="inlineStr">
         <is>
           <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113170115-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>5206756.182082118</v>
+      </c>
+      <c r="B82" t="n">
+        <v>26724.85275644315</v>
+      </c>
+      <c r="C82" t="n">
+        <v>3514.625425920614</v>
+      </c>
+      <c r="D82" t="n">
+        <v>9709.010080617943</v>
+      </c>
+      <c r="E82" t="n">
+        <v>2.207771026688302</v>
+      </c>
+      <c r="F82" t="n">
+        <v>36433.86283706109</v>
+      </c>
+      <c r="G82" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="H82" t="n">
+        <v>388450.9431906988</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" t="n">
+        <v>5206756.182082118</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0</v>
+      </c>
+      <c r="O82" t="n">
+        <v>0</v>
+      </c>
+      <c r="P82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>0</v>
+      </c>
+      <c r="R82" t="n">
+        <v>0</v>
+      </c>
+      <c r="S82" t="n">
+        <v>0</v>
+      </c>
+      <c r="T82" t="n">
+        <v>0</v>
+      </c>
+      <c r="U82" t="n">
+        <v>0</v>
+      </c>
+      <c r="V82" t="n">
+        <v>0.06699991226196289</v>
+      </c>
+      <c r="W82" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="X82" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="Y82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB82" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC82" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD82" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE82" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113184144-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>1431857.950072582</v>
+      </c>
+      <c r="B83" t="n">
+        <v>26724.85275644315</v>
+      </c>
+      <c r="C83" t="n">
+        <v>3514.625425920614</v>
+      </c>
+      <c r="D83" t="n">
+        <v>9709.010080617943</v>
+      </c>
+      <c r="E83" t="n">
+        <v>2.207771026688302</v>
+      </c>
+      <c r="F83" t="n">
+        <v>36433.86283706109</v>
+      </c>
+      <c r="G83" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="H83" t="n">
+        <v>388450.9431906988</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" t="n">
+        <v>1431857.950072582</v>
+      </c>
+      <c r="N83" t="n">
+        <v>0</v>
+      </c>
+      <c r="O83" t="n">
+        <v>0</v>
+      </c>
+      <c r="P83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>0</v>
+      </c>
+      <c r="R83" t="n">
+        <v>0</v>
+      </c>
+      <c r="S83" t="n">
+        <v>0</v>
+      </c>
+      <c r="T83" t="n">
+        <v>0</v>
+      </c>
+      <c r="U83" t="n">
+        <v>0</v>
+      </c>
+      <c r="V83" t="n">
+        <v>0.03799986839294434</v>
+      </c>
+      <c r="W83" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="X83" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="Y83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB83" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC83" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD83" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE83" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113184415-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>1041351.236416423</v>
+      </c>
+      <c r="B84" t="n">
+        <v>26724.85275644315</v>
+      </c>
+      <c r="C84" t="n">
+        <v>3514.625425920614</v>
+      </c>
+      <c r="D84" t="n">
+        <v>9709.010080617943</v>
+      </c>
+      <c r="E84" t="n">
+        <v>2.207771026688302</v>
+      </c>
+      <c r="F84" t="n">
+        <v>36433.86283706109</v>
+      </c>
+      <c r="G84" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="H84" t="n">
+        <v>388450.9431906988</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" t="n">
+        <v>1041351.236416423</v>
+      </c>
+      <c r="N84" t="n">
+        <v>0</v>
+      </c>
+      <c r="O84" t="n">
+        <v>0</v>
+      </c>
+      <c r="P84" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>0</v>
+      </c>
+      <c r="R84" t="n">
+        <v>0</v>
+      </c>
+      <c r="S84" t="n">
+        <v>0</v>
+      </c>
+      <c r="T84" t="n">
+        <v>0</v>
+      </c>
+      <c r="U84" t="n">
+        <v>0</v>
+      </c>
+      <c r="V84" t="n">
+        <v>0.03800010681152344</v>
+      </c>
+      <c r="W84" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="X84" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="Y84" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB84" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD84" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE84" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113184543-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>911182.33186437</v>
+      </c>
+      <c r="B85" t="n">
+        <v>26724.85275644315</v>
+      </c>
+      <c r="C85" t="n">
+        <v>3514.625425920614</v>
+      </c>
+      <c r="D85" t="n">
+        <v>9709.010080617943</v>
+      </c>
+      <c r="E85" t="n">
+        <v>2.207771026688302</v>
+      </c>
+      <c r="F85" t="n">
+        <v>36433.86283706109</v>
+      </c>
+      <c r="G85" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="H85" t="n">
+        <v>388450.9431906988</v>
+      </c>
+      <c r="I85" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" t="n">
+        <v>911182.33186437</v>
+      </c>
+      <c r="N85" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0</v>
+      </c>
+      <c r="P85" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>0</v>
+      </c>
+      <c r="R85" t="n">
+        <v>0</v>
+      </c>
+      <c r="S85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T85" t="n">
+        <v>0</v>
+      </c>
+      <c r="U85" t="n">
+        <v>0</v>
+      </c>
+      <c r="V85" t="n">
+        <v>0.05200004577636719</v>
+      </c>
+      <c r="W85" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="X85" t="n">
+        <v>3516.833196947302</v>
+      </c>
+      <c r="Y85" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA85" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB85" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC85" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD85" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE85" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113184701-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>833080.9891331382</v>
+      </c>
+      <c r="B86" t="n">
+        <v>26776.95315533437</v>
+      </c>
+      <c r="C86" t="n">
+        <v>3663.489068421782</v>
+      </c>
+      <c r="D86" t="n">
+        <v>9727.926776845998</v>
+      </c>
+      <c r="E86" t="n">
+        <v>3.468549727957493</v>
+      </c>
+      <c r="F86" t="n">
+        <v>36504.87993218037</v>
+      </c>
+      <c r="G86" t="n">
+        <v>3666.957618149739</v>
+      </c>
+      <c r="H86" t="n">
+        <v>388188.341497608</v>
+      </c>
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" t="n">
+        <v>833080.9891331382</v>
+      </c>
+      <c r="N86" t="n">
+        <v>0</v>
+      </c>
+      <c r="O86" t="n">
+        <v>0</v>
+      </c>
+      <c r="P86" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>0</v>
+      </c>
+      <c r="R86" t="n">
+        <v>0</v>
+      </c>
+      <c r="S86" t="n">
+        <v>0</v>
+      </c>
+      <c r="T86" t="n">
+        <v>0</v>
+      </c>
+      <c r="U86" t="n">
+        <v>0</v>
+      </c>
+      <c r="V86" t="n">
+        <v>0.05699992179870605</v>
+      </c>
+      <c r="W86" t="n">
+        <v>3666.957618149739</v>
+      </c>
+      <c r="X86" t="n">
+        <v>3666.957618149739</v>
+      </c>
+      <c r="Y86" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z86" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA86" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB86" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC86" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD86" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE86" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113184823-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>781013.4273123173</v>
+      </c>
+      <c r="B87" t="n">
+        <v>25146.98458303148</v>
+      </c>
+      <c r="C87" t="n">
+        <v>4052.094415821957</v>
+      </c>
+      <c r="D87" t="n">
+        <v>9136.115178476019</v>
+      </c>
+      <c r="E87" t="n">
+        <v>4.949996077802806</v>
+      </c>
+      <c r="F87" t="n">
+        <v>34283.0997615075</v>
+      </c>
+      <c r="G87" t="n">
+        <v>4057.04441189976</v>
+      </c>
+      <c r="H87" t="n">
+        <v>389127.8107377011</v>
+      </c>
+      <c r="I87" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" t="n">
+        <v>781013.4273123173</v>
+      </c>
+      <c r="N87" t="n">
+        <v>0</v>
+      </c>
+      <c r="O87" t="n">
+        <v>0</v>
+      </c>
+      <c r="P87" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>0</v>
+      </c>
+      <c r="R87" t="n">
+        <v>0</v>
+      </c>
+      <c r="S87" t="n">
+        <v>0</v>
+      </c>
+      <c r="T87" t="n">
+        <v>0</v>
+      </c>
+      <c r="U87" t="n">
+        <v>0</v>
+      </c>
+      <c r="V87" t="n">
+        <v>0.03700017929077148</v>
+      </c>
+      <c r="W87" t="n">
+        <v>4057.04441189976</v>
+      </c>
+      <c r="X87" t="n">
+        <v>4057.04441189976</v>
+      </c>
+      <c r="Y87" t="n">
+        <v>4.547473508864641e-13</v>
+      </c>
+      <c r="Z87" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB87" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC87" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD87" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE87" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113184937-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>728945.8654914962</v>
+      </c>
+      <c r="B88" t="n">
+        <v>19933.79296549723</v>
+      </c>
+      <c r="C88" t="n">
+        <v>5369.651718085902</v>
+      </c>
+      <c r="D88" t="n">
+        <v>7243.301221073767</v>
+      </c>
+      <c r="E88" t="n">
+        <v>7.377807991047177</v>
+      </c>
+      <c r="F88" t="n">
+        <v>27177.094186571</v>
+      </c>
+      <c r="G88" t="n">
+        <v>5377.029526076949</v>
+      </c>
+      <c r="H88" t="n">
+        <v>392514.6067005237</v>
+      </c>
+      <c r="I88" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" t="n">
+        <v>728945.8654914962</v>
+      </c>
+      <c r="N88" t="n">
+        <v>0</v>
+      </c>
+      <c r="O88" t="n">
+        <v>0</v>
+      </c>
+      <c r="P88" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>0</v>
+      </c>
+      <c r="R88" t="n">
+        <v>0</v>
+      </c>
+      <c r="S88" t="n">
+        <v>0</v>
+      </c>
+      <c r="T88" t="n">
+        <v>0</v>
+      </c>
+      <c r="U88" t="n">
+        <v>0</v>
+      </c>
+      <c r="V88" t="n">
+        <v>0.03099989891052246</v>
+      </c>
+      <c r="W88" t="n">
+        <v>5377.029526076948</v>
+      </c>
+      <c r="X88" t="n">
+        <v>5377.029526076949</v>
+      </c>
+      <c r="Y88" t="n">
+        <v>9.094947017729282e-13</v>
+      </c>
+      <c r="Z88" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA88" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB88" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC88" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD88" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE88" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113185231-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>387778799.0272403</v>
+      </c>
+      <c r="B89" t="n">
+        <v>33946254.17293455</v>
+      </c>
+      <c r="C89" t="n">
+        <v>7813218.524940382</v>
+      </c>
+      <c r="D89" t="n">
+        <v>12329506.84931507</v>
+      </c>
+      <c r="E89" t="n">
+        <v>1988.169409936008</v>
+      </c>
+      <c r="F89" t="n">
+        <v>46275761.02224962</v>
+      </c>
+      <c r="G89" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="H89" t="n">
+        <v>308546019.908245</v>
+      </c>
+      <c r="I89" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" t="n">
+        <v>387778799.0272403</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0</v>
+      </c>
+      <c r="O89" t="n">
+        <v>0</v>
+      </c>
+      <c r="P89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>0</v>
+      </c>
+      <c r="R89" t="n">
+        <v>0</v>
+      </c>
+      <c r="S89" t="n">
+        <v>0</v>
+      </c>
+      <c r="T89" t="n">
+        <v>0</v>
+      </c>
+      <c r="U89" t="n">
+        <v>0</v>
+      </c>
+      <c r="V89" t="n">
+        <v>74.93600010871887</v>
+      </c>
+      <c r="W89" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="X89" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="Y89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z89" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA89" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB89" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC89" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD89" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE89" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113185900-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>387869108.0266845</v>
+      </c>
+      <c r="B90" t="n">
+        <v>33946254.17293455</v>
+      </c>
+      <c r="C90" t="n">
+        <v>7813218.524940382</v>
+      </c>
+      <c r="D90" t="n">
+        <v>12329506.84931507</v>
+      </c>
+      <c r="E90" t="n">
+        <v>1988.169409936009</v>
+      </c>
+      <c r="F90" t="n">
+        <v>46275761.02224962</v>
+      </c>
+      <c r="G90" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="H90" t="n">
+        <v>308636328.9076893</v>
+      </c>
+      <c r="I90" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" t="n">
+        <v>387869108.0266845</v>
+      </c>
+      <c r="N90" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" t="n">
+        <v>0</v>
+      </c>
+      <c r="P90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>0</v>
+      </c>
+      <c r="R90" t="n">
+        <v>0</v>
+      </c>
+      <c r="S90" t="n">
+        <v>0</v>
+      </c>
+      <c r="T90" t="n">
+        <v>0</v>
+      </c>
+      <c r="U90" t="n">
+        <v>0</v>
+      </c>
+      <c r="V90" t="n">
+        <v>36.47199988365173</v>
+      </c>
+      <c r="W90" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="X90" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="Y90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z90" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>supply_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB90" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC90" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD90" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE90" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113190501-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>781013.4273123173</v>
+      </c>
+      <c r="B91" t="n">
+        <v>25146.98458303148</v>
+      </c>
+      <c r="C91" t="n">
+        <v>4052.094415821957</v>
+      </c>
+      <c r="D91" t="n">
+        <v>9136.115178476019</v>
+      </c>
+      <c r="E91" t="n">
+        <v>4.949996077802806</v>
+      </c>
+      <c r="F91" t="n">
+        <v>34283.0997615075</v>
+      </c>
+      <c r="G91" t="n">
+        <v>4057.04441189976</v>
+      </c>
+      <c r="H91" t="n">
+        <v>389127.8107377011</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="n">
+        <v>781013.4273123173</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>0</v>
+      </c>
+      <c r="R91" t="n">
+        <v>0</v>
+      </c>
+      <c r="S91" t="n">
+        <v>0</v>
+      </c>
+      <c r="T91" t="n">
+        <v>0</v>
+      </c>
+      <c r="U91" t="n">
+        <v>0</v>
+      </c>
+      <c r="V91" t="n">
+        <v>0.03100013732910156</v>
+      </c>
+      <c r="W91" t="n">
+        <v>4057.04441189976</v>
+      </c>
+      <c r="X91" t="n">
+        <v>4057.04441189976</v>
+      </c>
+      <c r="Y91" t="n">
+        <v>4.547473508864641e-13</v>
+      </c>
+      <c r="Z91" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA91" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB91" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC91" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD91" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE91" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113191116-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>387778799.0272403</v>
+      </c>
+      <c r="B92" t="n">
+        <v>33946254.17293455</v>
+      </c>
+      <c r="C92" t="n">
+        <v>7813218.524940382</v>
+      </c>
+      <c r="D92" t="n">
+        <v>12329506.84931507</v>
+      </c>
+      <c r="E92" t="n">
+        <v>1988.169409936008</v>
+      </c>
+      <c r="F92" t="n">
+        <v>46275761.02224962</v>
+      </c>
+      <c r="G92" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="H92" t="n">
+        <v>308546019.908245</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="n">
+        <v>0</v>
+      </c>
+      <c r="M92" t="n">
+        <v>387778799.0272403</v>
+      </c>
+      <c r="N92" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0</v>
+      </c>
+      <c r="P92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>0</v>
+      </c>
+      <c r="R92" t="n">
+        <v>0</v>
+      </c>
+      <c r="S92" t="n">
+        <v>0</v>
+      </c>
+      <c r="T92" t="n">
+        <v>0</v>
+      </c>
+      <c r="U92" t="n">
+        <v>0</v>
+      </c>
+      <c r="V92" t="n">
+        <v>70.68700003623962</v>
+      </c>
+      <c r="W92" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="X92" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="Y92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z92" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA92" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB92" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC92" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD92" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE92" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113191420-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>4294683461.202195</v>
+      </c>
+      <c r="B93" t="n">
+        <v>399689766.8748745</v>
+      </c>
+      <c r="C93" t="n">
+        <v>124754801.8117265</v>
+      </c>
+      <c r="D93" t="n">
+        <v>145170000</v>
+      </c>
+      <c r="E93" t="n">
+        <v>24515.8938377547</v>
+      </c>
+      <c r="F93" t="n">
+        <v>544859766.8748745</v>
+      </c>
+      <c r="G93" t="n">
+        <v>124779317.7055643</v>
+      </c>
+      <c r="H93" t="n">
+        <v>3536810305.950909</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" t="n">
+        <v>4294683461.202195</v>
+      </c>
+      <c r="N93" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0</v>
+      </c>
+      <c r="P93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>0</v>
+      </c>
+      <c r="R93" t="n">
+        <v>0</v>
+      </c>
+      <c r="S93" t="n">
+        <v>0</v>
+      </c>
+      <c r="T93" t="n">
+        <v>0</v>
+      </c>
+      <c r="U93" t="n">
+        <v>0</v>
+      </c>
+      <c r="V93" t="n">
+        <v>2451.382999897003</v>
+      </c>
+      <c r="W93" t="n">
+        <v>124779317.7054293</v>
+      </c>
+      <c r="X93" t="n">
+        <v>124779317.7055643</v>
+      </c>
+      <c r="Y93" t="n">
+        <v>0.0001350045204162598</v>
+      </c>
+      <c r="Z93" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA93" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB93" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC93" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD93" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE93" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251113193303-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>387778799.0272403</v>
+      </c>
+      <c r="B94" t="n">
+        <v>33946254.17293455</v>
+      </c>
+      <c r="C94" t="n">
+        <v>7813218.524940382</v>
+      </c>
+      <c r="D94" t="n">
+        <v>12329506.84931507</v>
+      </c>
+      <c r="E94" t="n">
+        <v>1988.169409936008</v>
+      </c>
+      <c r="F94" t="n">
+        <v>46275761.02224962</v>
+      </c>
+      <c r="G94" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="H94" t="n">
+        <v>308546019.908245</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" t="n">
+        <v>0</v>
+      </c>
+      <c r="M94" t="n">
+        <v>387778799.0272403</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>0</v>
+      </c>
+      <c r="R94" t="n">
+        <v>0</v>
+      </c>
+      <c r="S94" t="n">
+        <v>0</v>
+      </c>
+      <c r="T94" t="n">
+        <v>0</v>
+      </c>
+      <c r="U94" t="n">
+        <v>0</v>
+      </c>
+      <c r="V94" t="n">
+        <v>123.7799999713898</v>
+      </c>
+      <c r="W94" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="X94" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="Y94" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z94" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB94" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC94" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD94" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE94" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114082700-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>387778799.0272403</v>
+      </c>
+      <c r="B95" t="n">
+        <v>33946254.17293455</v>
+      </c>
+      <c r="C95" t="n">
+        <v>7813218.524940382</v>
+      </c>
+      <c r="D95" t="n">
+        <v>12329506.84931507</v>
+      </c>
+      <c r="E95" t="n">
+        <v>1988.169409936008</v>
+      </c>
+      <c r="F95" t="n">
+        <v>46275761.02224962</v>
+      </c>
+      <c r="G95" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="H95" t="n">
+        <v>308546019.908245</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" t="n">
+        <v>387778799.0272403</v>
+      </c>
+      <c r="N95" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>0</v>
+      </c>
+      <c r="R95" t="n">
+        <v>0</v>
+      </c>
+      <c r="S95" t="n">
+        <v>0</v>
+      </c>
+      <c r="T95" t="n">
+        <v>0</v>
+      </c>
+      <c r="U95" t="n">
+        <v>0</v>
+      </c>
+      <c r="V95" t="n">
+        <v>150.4900000095367</v>
+      </c>
+      <c r="W95" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="X95" t="n">
+        <v>7815206.694350318</v>
+      </c>
+      <c r="Y95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB95" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC95" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD95" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE95" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114083543-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>447042207.9459601</v>
+      </c>
+      <c r="B96" t="n">
+        <v>77380243.00660133</v>
+      </c>
+      <c r="C96" t="n">
+        <v>318262.3830684706</v>
+      </c>
+      <c r="D96" t="n">
+        <v>28099589.04109589</v>
+      </c>
+      <c r="E96" t="n">
+        <v>466.9811862896512</v>
+      </c>
+      <c r="F96" t="n">
+        <v>105479832.0476972</v>
+      </c>
+      <c r="G96" t="n">
+        <v>318729.3642547603</v>
+      </c>
+      <c r="H96" t="n">
+        <v>310500627.5020258</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" t="n">
+        <v>447042207.9459601</v>
+      </c>
+      <c r="N96" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>0</v>
+      </c>
+      <c r="R96" t="n">
+        <v>0</v>
+      </c>
+      <c r="S96" t="n">
+        <v>0</v>
+      </c>
+      <c r="T96" t="n">
+        <v>0</v>
+      </c>
+      <c r="U96" t="n">
+        <v>0</v>
+      </c>
+      <c r="V96" t="n">
+        <v>56.31800007820129</v>
+      </c>
+      <c r="W96" t="n">
+        <v>318729.3642547603</v>
+      </c>
+      <c r="X96" t="n">
+        <v>318729.3642547603</v>
+      </c>
+      <c r="Y96" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB96" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC96" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD96" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE96" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114085339-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>426421907.1799636</v>
+      </c>
+      <c r="B97" t="n">
+        <v>63401272.88219413</v>
+      </c>
+      <c r="C97" t="n">
+        <v>318262.3830684706</v>
+      </c>
+      <c r="D97" t="n">
+        <v>23024082.19178082</v>
+      </c>
+      <c r="E97" t="n">
+        <v>466.9811862896531</v>
+      </c>
+      <c r="F97" t="n">
+        <v>86425355.07397495</v>
+      </c>
+      <c r="G97" t="n">
+        <v>318729.3642547602</v>
+      </c>
+      <c r="H97" t="n">
+        <v>309685726.1543473</v>
+      </c>
+      <c r="I97" t="n">
+        <v>0</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" t="n">
+        <v>0</v>
+      </c>
+      <c r="M97" t="n">
+        <v>426421907.1799636</v>
+      </c>
+      <c r="N97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O97" t="n">
+        <v>0</v>
+      </c>
+      <c r="P97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>0</v>
+      </c>
+      <c r="R97" t="n">
+        <v>0</v>
+      </c>
+      <c r="S97" t="n">
+        <v>0</v>
+      </c>
+      <c r="T97" t="n">
+        <v>0</v>
+      </c>
+      <c r="U97" t="n">
+        <v>0</v>
+      </c>
+      <c r="V97" t="n">
+        <v>31.02900004386902</v>
+      </c>
+      <c r="W97" t="n">
+        <v>318729.3642547602</v>
+      </c>
+      <c r="X97" t="n">
+        <v>318729.3642547602</v>
+      </c>
+      <c r="Y97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB97" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC97" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD97" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE97" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114093759-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>4677650654.035797</v>
+      </c>
+      <c r="B98" t="n">
+        <v>746498858.12906</v>
+      </c>
+      <c r="C98" t="n">
+        <v>10997383.60314498</v>
+      </c>
+      <c r="D98" t="n">
+        <v>271090000</v>
+      </c>
+      <c r="E98" t="n">
+        <v>4863.46806870262</v>
+      </c>
+      <c r="F98" t="n">
+        <v>1017588858.12906</v>
+      </c>
+      <c r="G98" t="n">
+        <v>11002247.07121368</v>
+      </c>
+      <c r="H98" t="n">
+        <v>3547415621.393197</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0</v>
+      </c>
+      <c r="L98" t="n">
+        <v>0</v>
+      </c>
+      <c r="M98" t="n">
+        <v>4677650654.035797</v>
+      </c>
+      <c r="N98" t="n">
+        <v>0</v>
+      </c>
+      <c r="O98" t="n">
+        <v>0</v>
+      </c>
+      <c r="P98" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>0</v>
+      </c>
+      <c r="R98" t="n">
+        <v>0</v>
+      </c>
+      <c r="S98" t="n">
+        <v>0</v>
+      </c>
+      <c r="T98" t="n">
+        <v>0</v>
+      </c>
+      <c r="U98" t="n">
+        <v>0</v>
+      </c>
+      <c r="V98" t="n">
+        <v>795.6210000514984</v>
+      </c>
+      <c r="W98" t="n">
+        <v>11002247.07120266</v>
+      </c>
+      <c r="X98" t="n">
+        <v>11002247.07121368</v>
+      </c>
+      <c r="Y98" t="n">
+        <v>1.102499663829803e-05</v>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB98" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC98" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD98" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE98" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114100233-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>4760720292.095636</v>
+      </c>
+      <c r="B99" t="n">
+        <v>790566087.0050685</v>
+      </c>
+      <c r="C99" t="n">
+        <v>9478453.888726894</v>
+      </c>
+      <c r="D99" t="n">
+        <v>287090000</v>
+      </c>
+      <c r="E99" t="n">
+        <v>1390.049463288724</v>
+      </c>
+      <c r="F99" t="n">
+        <v>1077656087.005069</v>
+      </c>
+      <c r="G99" t="n">
+        <v>9479843.938190183</v>
+      </c>
+      <c r="H99" t="n">
+        <v>3571400765.836381</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" t="n">
+        <v>0</v>
+      </c>
+      <c r="M99" t="n">
+        <v>4760720292.095636</v>
+      </c>
+      <c r="N99" t="n">
+        <v>0</v>
+      </c>
+      <c r="O99" t="n">
+        <v>0</v>
+      </c>
+      <c r="P99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>0</v>
+      </c>
+      <c r="R99" t="n">
+        <v>0</v>
+      </c>
+      <c r="S99" t="n">
+        <v>0</v>
+      </c>
+      <c r="T99" t="n">
+        <v>0</v>
+      </c>
+      <c r="U99" t="n">
+        <v>0</v>
+      </c>
+      <c r="V99" t="n">
+        <v>849.0490000247955</v>
+      </c>
+      <c r="W99" t="n">
+        <v>9479843.938189447</v>
+      </c>
+      <c r="X99" t="n">
+        <v>9479843.938190183</v>
+      </c>
+      <c r="Y99" t="n">
+        <v>7.35744833946228e-07</v>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB99" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC99" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD99" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE99" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114104442-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>4743064870.58446</v>
+      </c>
+      <c r="B100" t="n">
+        <v>790566087.0050685</v>
+      </c>
+      <c r="C100" t="n">
+        <v>9510277.663202683</v>
+      </c>
+      <c r="D100" t="n">
+        <v>287090000</v>
+      </c>
+      <c r="E100" t="n">
+        <v>1390.049463288721</v>
+      </c>
+      <c r="F100" t="n">
+        <v>1077656087.005069</v>
+      </c>
+      <c r="G100" t="n">
+        <v>9511667.712665971</v>
+      </c>
+      <c r="H100" t="n">
+        <v>3566261720.477891</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0</v>
+      </c>
+      <c r="L100" t="n">
+        <v>0</v>
+      </c>
+      <c r="M100" t="n">
+        <v>4743064870.58446</v>
+      </c>
+      <c r="N100" t="n">
+        <v>0</v>
+      </c>
+      <c r="O100" t="n">
+        <v>0</v>
+      </c>
+      <c r="P100" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>0</v>
+      </c>
+      <c r="R100" t="n">
+        <v>0</v>
+      </c>
+      <c r="S100" t="n">
+        <v>0</v>
+      </c>
+      <c r="T100" t="n">
+        <v>0</v>
+      </c>
+      <c r="U100" t="n">
+        <v>0</v>
+      </c>
+      <c r="V100" t="n">
+        <v>592.5439999103546</v>
+      </c>
+      <c r="W100" t="n">
+        <v>9484743.620351544</v>
+      </c>
+      <c r="X100" t="n">
+        <v>9511667.712665971</v>
+      </c>
+      <c r="Y100" t="n">
+        <v>26924.09231442772</v>
+      </c>
+      <c r="Z100" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA100" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB100" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC100" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD100" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE100" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114112810-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>4641334790.052398</v>
+      </c>
+      <c r="B101" t="n">
+        <v>497406181.0224904</v>
+      </c>
+      <c r="C101" t="n">
+        <v>8191807.776157273</v>
+      </c>
+      <c r="D101" t="n">
+        <v>180649032.2062313</v>
+      </c>
+      <c r="E101" t="n">
+        <v>1.520455075121863</v>
+      </c>
+      <c r="F101" t="n">
+        <v>678055213.2287217</v>
+      </c>
+      <c r="G101" t="n">
+        <v>8191809.296612348</v>
+      </c>
+      <c r="H101" t="n">
+        <v>3951066977.691289</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" t="n">
+        <v>0</v>
+      </c>
+      <c r="M101" t="n">
+        <v>4641334790.052398</v>
+      </c>
+      <c r="N101" t="n">
+        <v>0</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0</v>
+      </c>
+      <c r="P101" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>0</v>
+      </c>
+      <c r="R101" t="n">
+        <v>0</v>
+      </c>
+      <c r="S101" t="n">
+        <v>0</v>
+      </c>
+      <c r="T101" t="n">
+        <v>0</v>
+      </c>
+      <c r="U101" t="n">
+        <v>0</v>
+      </c>
+      <c r="V101" t="n">
+        <v>829.6400001049042</v>
+      </c>
+      <c r="W101" t="n">
+        <v>8174031.734872591</v>
+      </c>
+      <c r="X101" t="n">
+        <v>8191809.296612348</v>
+      </c>
+      <c r="Y101" t="n">
+        <v>17777.56173975766</v>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA101" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB101" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC101" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD101" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE101" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114124047-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>5604557284.88429</v>
+      </c>
+      <c r="B102" t="n">
+        <v>497406181.0224904</v>
+      </c>
+      <c r="C102" t="n">
+        <v>8191807.776157273</v>
+      </c>
+      <c r="D102" t="n">
+        <v>180649032.2062313</v>
+      </c>
+      <c r="E102" t="n">
+        <v>1.520455075121863</v>
+      </c>
+      <c r="F102" t="n">
+        <v>678055213.2287217</v>
+      </c>
+      <c r="G102" t="n">
+        <v>8191809.296612348</v>
+      </c>
+      <c r="H102" t="n">
+        <v>4914289472.523181</v>
+      </c>
+      <c r="I102" t="n">
+        <v>0</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0</v>
+      </c>
+      <c r="L102" t="n">
+        <v>0</v>
+      </c>
+      <c r="M102" t="n">
+        <v>5604557284.88429</v>
+      </c>
+      <c r="N102" t="n">
+        <v>0</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0</v>
+      </c>
+      <c r="P102" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>0</v>
+      </c>
+      <c r="R102" t="n">
+        <v>0</v>
+      </c>
+      <c r="S102" t="n">
+        <v>0</v>
+      </c>
+      <c r="T102" t="n">
+        <v>0</v>
+      </c>
+      <c r="U102" t="n">
+        <v>0</v>
+      </c>
+      <c r="V102" t="n">
+        <v>797.3139998912811</v>
+      </c>
+      <c r="W102" t="n">
+        <v>8174031.734872591</v>
+      </c>
+      <c r="X102" t="n">
+        <v>8191809.296612348</v>
+      </c>
+      <c r="Y102" t="n">
+        <v>17777.56173975766</v>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA102" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB102" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC102" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD102" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE102" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114132059-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>5564309658.803686</v>
+      </c>
+      <c r="B103" t="n">
+        <v>790566087.0050685</v>
+      </c>
+      <c r="C103" t="n">
+        <v>9510277.663202683</v>
+      </c>
+      <c r="D103" t="n">
+        <v>287090000</v>
+      </c>
+      <c r="E103" t="n">
+        <v>1390.049463288716</v>
+      </c>
+      <c r="F103" t="n">
+        <v>1077656087.005069</v>
+      </c>
+      <c r="G103" t="n">
+        <v>9511667.712665971</v>
+      </c>
+      <c r="H103" t="n">
+        <v>4387365161.58816</v>
+      </c>
+      <c r="I103" t="n">
+        <v>0</v>
+      </c>
+      <c r="J103" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" t="n">
+        <v>0</v>
+      </c>
+      <c r="M103" t="n">
+        <v>5564309658.803686</v>
+      </c>
+      <c r="N103" t="n">
+        <v>0</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0</v>
+      </c>
+      <c r="P103" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>0</v>
+      </c>
+      <c r="R103" t="n">
+        <v>0</v>
+      </c>
+      <c r="S103" t="n">
+        <v>0</v>
+      </c>
+      <c r="T103" t="n">
+        <v>0</v>
+      </c>
+      <c r="U103" t="n">
+        <v>0</v>
+      </c>
+      <c r="V103" t="n">
+        <v>979.8439998626709</v>
+      </c>
+      <c r="W103" t="n">
+        <v>9484743.620351553</v>
+      </c>
+      <c r="X103" t="n">
+        <v>9511667.712665971</v>
+      </c>
+      <c r="Y103" t="n">
+        <v>26924.09231441841</v>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB103" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC103" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD103" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE103" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114140239-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>5022354205.054915</v>
+      </c>
+      <c r="B104" t="n">
+        <v>702431629.2530516</v>
+      </c>
+      <c r="C104" t="n">
+        <v>15720383.87663246</v>
+      </c>
+      <c r="D104" t="n">
+        <v>255090000</v>
+      </c>
+      <c r="E104" t="n">
+        <v>14128.24588486611</v>
+      </c>
+      <c r="F104" t="n">
+        <v>957521629.2530516</v>
+      </c>
+      <c r="G104" t="n">
+        <v>15734512.12251733</v>
+      </c>
+      <c r="H104" t="n">
+        <v>3964498423.850807</v>
+      </c>
+      <c r="I104" t="n">
+        <v>0</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0</v>
+      </c>
+      <c r="L104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M104" t="n">
+        <v>5022354205.054915</v>
+      </c>
+      <c r="N104" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" t="n">
+        <v>0</v>
+      </c>
+      <c r="P104" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>0</v>
+      </c>
+      <c r="R104" t="n">
+        <v>0</v>
+      </c>
+      <c r="S104" t="n">
+        <v>0</v>
+      </c>
+      <c r="T104" t="n">
+        <v>0</v>
+      </c>
+      <c r="U104" t="n">
+        <v>0</v>
+      </c>
+      <c r="V104" t="n">
+        <v>1999.912999868393</v>
+      </c>
+      <c r="W104" t="n">
+        <v>15659201.78827695</v>
+      </c>
+      <c r="X104" t="n">
+        <v>15734512.12251733</v>
+      </c>
+      <c r="Y104" t="n">
+        <v>75310.33424037509</v>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>distance_willingness_to_pay</t>
+        </is>
+      </c>
+      <c r="AB104" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AC104" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD104" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AE104" t="inlineStr">
+        <is>
+          <t>Z:\AdOpT-NET0-RegToNation\generic_node_optimization\userData\20251114144507-1</t>
         </is>
       </c>
     </row>

</xml_diff>